<commit_message>
Refactor photo and document upload handling across multiple pages
- Updated ActivitiesPage to allow multiple photo uploads at once, enforcing a maximum limit of 10 photos and providing user feedback on upload status.
- Enhanced FinancePage with field-level validation for donations and expenses, including required fields and error messages. Added support for multiple file uploads for receipts and vouchers.
- Modified MeetingsPage to support batch uploads for photos and documents, with a limit of 10 photos and 5 documents, ensuring user feedback on upload status.
- Introduced utility constants for maximum upload limits to maintain consistency across components.
</commit_message>
<xml_diff>
--- a/PNAP-Punjab-Sindh-Setup-DETAILED.xlsx
+++ b/PNAP-Punjab-Sindh-Setup-DETAILED.xlsx
@@ -1,14 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C591A4-AD3E-4408-A043-27D132447020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Overview" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Admin Credentials" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Members" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Org Structure" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Role Assignments" state="visible" r:id="rId8"/>
+    <sheet name="Overview" sheetId="1" r:id="rId1"/>
+    <sheet name="Admin Credentials" sheetId="2" r:id="rId2"/>
+    <sheet name="Members" sheetId="3" r:id="rId3"/>
+    <sheet name="Org Structure" sheetId="4" r:id="rId4"/>
+    <sheet name="Role Assignments" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -2081,18 +2085,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="4">
@@ -2469,9 +2475,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2483,7 +2489,7 @@
     <col min="8" max="8" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2509,7 +2515,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -2535,7 +2541,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2562,16 +2568,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:H1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -2580,7 +2586,7 @@
     <col min="5" max="5" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -2597,7 +2603,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -2614,7 +2620,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2631,7 +2637,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>25</v>
       </c>
@@ -2648,7 +2654,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -2665,7 +2671,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -2682,7 +2688,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2699,7 +2705,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -2716,7 +2722,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -2733,7 +2739,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
@@ -2750,7 +2756,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -2767,7 +2773,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>25</v>
       </c>
@@ -2784,7 +2790,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -2801,7 +2807,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>25</v>
       </c>
@@ -2818,7 +2824,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -2835,7 +2841,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2852,7 +2858,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -2869,7 +2875,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>25</v>
       </c>
@@ -2886,7 +2892,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -2903,7 +2909,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2920,7 +2926,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -2937,7 +2943,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>25</v>
       </c>
@@ -2954,7 +2960,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>25</v>
       </c>
@@ -2971,7 +2977,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>21</v>
       </c>
@@ -2988,7 +2994,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -3005,7 +3011,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>25</v>
       </c>
@@ -3022,7 +3028,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -3040,16 +3046,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T73"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -3069,7 +3075,7 @@
     <col min="20" max="20" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
@@ -3131,7 +3137,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>113</v>
       </c>
@@ -3193,7 +3199,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>130</v>
       </c>
@@ -3255,7 +3261,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>139</v>
       </c>
@@ -3317,7 +3323,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>147</v>
       </c>
@@ -3379,7 +3385,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>155</v>
       </c>
@@ -3441,7 +3447,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>166</v>
       </c>
@@ -3503,7 +3509,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>174</v>
       </c>
@@ -3565,7 +3571,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>183</v>
       </c>
@@ -3627,7 +3633,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>190</v>
       </c>
@@ -3689,7 +3695,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>200</v>
       </c>
@@ -3751,7 +3757,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>207</v>
       </c>
@@ -3813,7 +3819,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>214</v>
       </c>
@@ -3875,7 +3881,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>221</v>
       </c>
@@ -3937,7 +3943,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>232</v>
       </c>
@@ -3999,7 +4005,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="16" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>238</v>
       </c>
@@ -4061,7 +4067,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>246</v>
       </c>
@@ -4123,7 +4129,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>253</v>
       </c>
@@ -4185,7 +4191,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>263</v>
       </c>
@@ -4247,7 +4253,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="20" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>270</v>
       </c>
@@ -4309,7 +4315,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>278</v>
       </c>
@@ -4371,7 +4377,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="22" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>284</v>
       </c>
@@ -4433,7 +4439,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>294</v>
       </c>
@@ -4495,7 +4501,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>301</v>
       </c>
@@ -4557,7 +4563,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>308</v>
       </c>
@@ -4619,7 +4625,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="26" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>315</v>
       </c>
@@ -4681,7 +4687,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>325</v>
       </c>
@@ -4743,7 +4749,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>331</v>
       </c>
@@ -4805,7 +4811,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>337</v>
       </c>
@@ -4867,7 +4873,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>343</v>
       </c>
@@ -4929,7 +4935,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>352</v>
       </c>
@@ -4991,7 +4997,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>357</v>
       </c>
@@ -5053,7 +5059,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>364</v>
       </c>
@@ -5115,7 +5121,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>370</v>
       </c>
@@ -5177,7 +5183,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>379</v>
       </c>
@@ -5239,7 +5245,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>385</v>
       </c>
@@ -5301,7 +5307,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>392</v>
       </c>
@@ -5363,7 +5369,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>397</v>
       </c>
@@ -5425,7 +5431,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>407</v>
       </c>
@@ -5487,7 +5493,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="40" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>413</v>
       </c>
@@ -5549,7 +5555,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>419</v>
       </c>
@@ -5611,7 +5617,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="42" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>425</v>
       </c>
@@ -5673,7 +5679,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>434</v>
       </c>
@@ -5735,7 +5741,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="44" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>439</v>
       </c>
@@ -5797,7 +5803,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>446</v>
       </c>
@@ -5859,7 +5865,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="46" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>452</v>
       </c>
@@ -5921,7 +5927,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>461</v>
       </c>
@@ -5983,7 +5989,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="48" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>466</v>
       </c>
@@ -6045,7 +6051,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>473</v>
       </c>
@@ -6107,7 +6113,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="50" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>478</v>
       </c>
@@ -6169,7 +6175,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>488</v>
       </c>
@@ -6231,7 +6237,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="52" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>494</v>
       </c>
@@ -6293,7 +6299,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>500</v>
       </c>
@@ -6355,7 +6361,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="54" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>506</v>
       </c>
@@ -6417,7 +6423,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>515</v>
       </c>
@@ -6479,7 +6485,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="56" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>521</v>
       </c>
@@ -6541,7 +6547,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>527</v>
       </c>
@@ -6603,7 +6609,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="58" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>533</v>
       </c>
@@ -6665,7 +6671,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>542</v>
       </c>
@@ -6727,7 +6733,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="60" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>547</v>
       </c>
@@ -6789,7 +6795,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>554</v>
       </c>
@@ -6851,7 +6857,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="62" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>559</v>
       </c>
@@ -6913,7 +6919,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>569</v>
       </c>
@@ -6975,7 +6981,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="64" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>575</v>
       </c>
@@ -7037,7 +7043,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>581</v>
       </c>
@@ -7099,7 +7105,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="66" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>587</v>
       </c>
@@ -7161,7 +7167,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>596</v>
       </c>
@@ -7223,7 +7229,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="68" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>601</v>
       </c>
@@ -7285,7 +7291,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>608</v>
       </c>
@@ -7347,7 +7353,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="70" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>614</v>
       </c>
@@ -7409,7 +7415,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>624</v>
       </c>
@@ -7471,7 +7477,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="72" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>629</v>
       </c>
@@ -7533,7 +7539,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>636</v>
       </c>
@@ -7596,16 +7602,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:T1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -7619,7 +7625,7 @@
     <col min="11" max="11" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7654,7 +7660,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
@@ -7689,7 +7695,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -7724,7 +7730,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -7759,7 +7765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -7794,7 +7800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -7829,7 +7835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -7864,7 +7870,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -7899,7 +7905,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -7934,7 +7940,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -7969,7 +7975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
@@ -8004,7 +8010,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
@@ -8039,7 +8045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>8</v>
       </c>
@@ -8074,7 +8080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
@@ -8109,7 +8115,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>8</v>
       </c>
@@ -8144,7 +8150,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
@@ -8179,7 +8185,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -8214,7 +8220,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>8</v>
       </c>
@@ -8249,7 +8255,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -8284,7 +8290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>12</v>
       </c>
@@ -8319,7 +8325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>12</v>
       </c>
@@ -8354,7 +8360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>12</v>
       </c>
@@ -8389,7 +8395,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>12</v>
       </c>
@@ -8424,7 +8430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>12</v>
       </c>
@@ -8459,7 +8465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>12</v>
       </c>
@@ -8494,7 +8500,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>12</v>
       </c>
@@ -8529,7 +8535,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>12</v>
       </c>
@@ -8564,7 +8570,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>12</v>
       </c>
@@ -8599,7 +8605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>12</v>
       </c>
@@ -8634,7 +8640,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>12</v>
       </c>
@@ -8669,7 +8675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>12</v>
       </c>
@@ -8704,7 +8710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
@@ -8739,7 +8745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -8774,7 +8780,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>12</v>
       </c>
@@ -8809,7 +8815,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -8844,7 +8850,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>12</v>
       </c>
@@ -8879,7 +8885,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -8915,16 +8921,16 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:K1" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J73"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -8938,7 +8944,7 @@
     <col min="10" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
@@ -8970,7 +8976,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>113</v>
       </c>
@@ -9002,7 +9008,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>130</v>
       </c>
@@ -9034,7 +9040,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>139</v>
       </c>
@@ -9066,7 +9072,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>147</v>
       </c>
@@ -9098,7 +9104,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>155</v>
       </c>
@@ -9130,7 +9136,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>166</v>
       </c>
@@ -9162,7 +9168,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>174</v>
       </c>
@@ -9194,7 +9200,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>183</v>
       </c>
@@ -9226,7 +9232,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>190</v>
       </c>
@@ -9258,7 +9264,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>200</v>
       </c>
@@ -9290,7 +9296,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>207</v>
       </c>
@@ -9322,7 +9328,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>214</v>
       </c>
@@ -9354,7 +9360,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>221</v>
       </c>
@@ -9386,7 +9392,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>232</v>
       </c>
@@ -9418,7 +9424,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>238</v>
       </c>
@@ -9450,7 +9456,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>246</v>
       </c>
@@ -9482,7 +9488,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>253</v>
       </c>
@@ -9514,7 +9520,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>263</v>
       </c>
@@ -9546,7 +9552,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>270</v>
       </c>
@@ -9578,7 +9584,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>278</v>
       </c>
@@ -9610,7 +9616,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>284</v>
       </c>
@@ -9642,7 +9648,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>294</v>
       </c>
@@ -9674,7 +9680,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>301</v>
       </c>
@@ -9706,7 +9712,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>308</v>
       </c>
@@ -9738,7 +9744,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>315</v>
       </c>
@@ -9770,7 +9776,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>325</v>
       </c>
@@ -9802,7 +9808,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>331</v>
       </c>
@@ -9834,7 +9840,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>337</v>
       </c>
@@ -9866,7 +9872,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>343</v>
       </c>
@@ -9898,7 +9904,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>352</v>
       </c>
@@ -9930,7 +9936,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>357</v>
       </c>
@@ -9962,7 +9968,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>364</v>
       </c>
@@ -9994,7 +10000,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>370</v>
       </c>
@@ -10026,7 +10032,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>379</v>
       </c>
@@ -10058,7 +10064,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>385</v>
       </c>
@@ -10090,7 +10096,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>392</v>
       </c>
@@ -10122,7 +10128,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>397</v>
       </c>
@@ -10154,7 +10160,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>407</v>
       </c>
@@ -10186,7 +10192,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>413</v>
       </c>
@@ -10218,7 +10224,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>419</v>
       </c>
@@ -10250,7 +10256,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>425</v>
       </c>
@@ -10282,7 +10288,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>434</v>
       </c>
@@ -10314,7 +10320,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>439</v>
       </c>
@@ -10346,7 +10352,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>446</v>
       </c>
@@ -10378,7 +10384,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>452</v>
       </c>
@@ -10410,7 +10416,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>461</v>
       </c>
@@ -10442,7 +10448,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>466</v>
       </c>
@@ -10474,7 +10480,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>473</v>
       </c>
@@ -10506,7 +10512,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>478</v>
       </c>
@@ -10538,7 +10544,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>488</v>
       </c>
@@ -10570,7 +10576,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="52" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>494</v>
       </c>
@@ -10602,7 +10608,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>500</v>
       </c>
@@ -10634,7 +10640,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="54" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>506</v>
       </c>
@@ -10666,7 +10672,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>515</v>
       </c>
@@ -10698,7 +10704,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>521</v>
       </c>
@@ -10730,7 +10736,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>527</v>
       </c>
@@ -10762,7 +10768,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>533</v>
       </c>
@@ -10794,7 +10800,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>542</v>
       </c>
@@ -10826,7 +10832,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>547</v>
       </c>
@@ -10858,7 +10864,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>554</v>
       </c>
@@ -10890,7 +10896,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>559</v>
       </c>
@@ -10922,7 +10928,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>569</v>
       </c>
@@ -10954,7 +10960,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="64" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>575</v>
       </c>
@@ -10986,7 +10992,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>581</v>
       </c>
@@ -11018,7 +11024,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="66" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>587</v>
       </c>
@@ -11050,7 +11056,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>596</v>
       </c>
@@ -11082,7 +11088,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>601</v>
       </c>
@@ -11114,7 +11120,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>608</v>
       </c>
@@ -11146,7 +11152,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="70" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>614</v>
       </c>
@@ -11178,7 +11184,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>624</v>
       </c>
@@ -11210,7 +11216,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="72" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>629</v>
       </c>
@@ -11242,7 +11248,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>636</v>
       </c>
@@ -11275,8 +11281,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J1" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>